<commit_message>
chore: 工作台自动同步 2026-09-12 00:32
</commit_message>
<xml_diff>
--- a/workbench/国产宠物药注册工作台.xlsx
+++ b/workbench/国产宠物药注册工作台.xlsx
@@ -8779,8 +8779,16 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>用于预防犬支气管败血波氏杆菌病</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>犬</t>
@@ -10497,8 +10505,16 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>用于检测猫嵌杯病毒荧光免疫层析法</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>猫</t>
@@ -10553,8 +10569,16 @@
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>用于检测犬细小病毒、猫细小病毒</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>犬、猫</t>

</xml_diff>

<commit_message>
chore: 工作台自动同步 2026-09-21 23:48
</commit_message>
<xml_diff>
--- a/workbench/国产宠物药注册工作台.xlsx
+++ b/workbench/国产宠物药注册工作台.xlsx
@@ -705,8 +705,16 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>用于敏感菌及支原体、衣原体、立克次体等引起的呼吸道、消化道感染（四环素类抗生素）。</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
@@ -757,8 +765,16 @@
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>用于相关疾病的治疗或预防（化药）</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>inferred</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
@@ -9011,8 +9027,16 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>用于预防猫鼻气管炎、杯状病毒病、泛白细胞减少症三联</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>猫</t>
@@ -10793,8 +10817,16 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>用于检测犬、猫狂犬病病毒抗体</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>犬、猫</t>
@@ -10849,8 +10881,16 @@
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>用于检测犬腺病毒Ⅰ型荧光</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>犬</t>
@@ -10905,8 +10945,16 @@
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>用于检测猫泛白细胞减少症病毒</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t>猫</t>

</xml_diff>

<commit_message>
chore: 工作台定时同步 2026-10-03 02:59
</commit_message>
<xml_diff>
--- a/workbench/国产宠物药注册工作台.xlsx
+++ b/workbench/国产宠物药注册工作台.xlsx
@@ -897,8 +897,16 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>用于预防犬细小病毒免疫球蛋白</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>犬</t>
@@ -953,8 +961,16 @@
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>用于抗炎、抗过敏及免疫抑制（糖皮质激素）。</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
@@ -11365,8 +11381,16 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>用于检测猫疱疹病毒1型</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>猫</t>
@@ -11421,8 +11445,16 @@
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>用于检测猫泛白细胞减少症病毒</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>猫</t>

</xml_diff>